<commit_message>
Initialize or update Git repository
</commit_message>
<xml_diff>
--- a/FigafIRTinfrastructure/IntegrationFlow/IRTHTTPtoProcessDirect/Documentation.xlsx
+++ b/FigafIRTinfrastructure/IntegrationFlow/IRTHTTPtoProcessDirect/Documentation.xlsx
@@ -314,7 +314,7 @@
     <t>SAP_ProfileId</t>
   </si>
   <si>
-    <t>sampledev(cpi-trial-alex)-&gt;sampleqa(cpi-trial-alex)</t>
+    <t>sampledev(trial-cpi-alex)-&gt;sampleqa(trial-cpi-alex)</t>
   </si>
   <si>
     <t>sampledev</t>
@@ -341,19 +341,19 @@
     <t>Not Required</t>
   </si>
   <si>
+    <t>Script</t>
+  </si>
+  <si>
+    <t>unwrap-figaf-headers.groovy</t>
+  </si>
+  <si>
+    <t>2026-07-13 06:55 AM</t>
+  </si>
+  <si>
     <t>IFlow Configuration</t>
   </si>
   <si>
     <t>IRTHTTPtoProcessDirect iflow configuration.json</t>
-  </si>
-  <si>
-    <t>2026-07-13 06:55 AM</t>
-  </si>
-  <si>
-    <t>Script</t>
-  </si>
-  <si>
-    <t>unwrap-figaf-headers.groovy</t>
   </si>
 </sst>
 </file>

</xml_diff>